<commit_message>
Update fin models: all 3 JK now target 20% net margin under FOT growth scenarios
Co-authored-by: kpetlin21-bot <kpetlin21-bot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/budget/output/Фин.модель — Астрид.xlsx
+++ b/budget/output/Фин.модель — Астрид.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Текущий бюджет" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="+30% ФОТ" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="+40% ФОТ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="+30% ФОТ → 20%" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="+40% ФОТ → 20%" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1594,7 +1594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1609,7 +1609,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Финансовая модель — Астрид  |  Сценарий: ФОТ +30%</t>
+          <t>Финансовая модель — Астрид  |  ФОТ +30%  →  цель ЧП 20%</t>
         </is>
       </c>
     </row>
@@ -1731,7 +1731,7 @@
         <v>2234664</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>3018477.555</v>
+        <v>4836736.082278481</v>
       </c>
     </row>
     <row r="7">
@@ -2212,28 +2212,28 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>ВАЛОВАЯ ПРИБЫЛЬ</t>
         </is>
       </c>
-      <c r="B28" s="14" t="n">
+      <c r="B28" s="8" t="n">
         <v>-419488</v>
       </c>
-      <c r="C28" s="14" t="n">
+      <c r="C28" s="8" t="n">
         <v>454070</v>
       </c>
-      <c r="D28" s="14" t="n">
+      <c r="D28" s="8" t="n">
         <v>-419488</v>
       </c>
-      <c r="E28" s="14" t="n">
+      <c r="E28" s="8" t="n">
         <v>28471</v>
       </c>
-      <c r="F28" s="14" t="n">
+      <c r="F28" s="8" t="n">
         <v>-356435</v>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>-319110.5449999999</v>
+      <c r="G28" s="8" t="n">
+        <v>1499147.982278481</v>
       </c>
     </row>
     <row r="29">
@@ -2249,7 +2249,7 @@
       <c r="F29" s="16" t="inlineStr"/>
       <c r="G29" s="16" t="inlineStr">
         <is>
-          <t>-10.6%</t>
+          <t>31.0%</t>
         </is>
       </c>
     </row>
@@ -2317,28 +2317,28 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>ОПЕРАЦИОННАЯ ПРИБЫЛЬ</t>
         </is>
       </c>
-      <c r="B33" s="14" t="n">
+      <c r="B33" s="8" t="n">
         <v>-475309</v>
       </c>
-      <c r="C33" s="14" t="n">
+      <c r="C33" s="8" t="n">
         <v>369151</v>
       </c>
-      <c r="D33" s="14" t="n">
+      <c r="D33" s="8" t="n">
         <v>-475309</v>
       </c>
-      <c r="E33" s="14" t="n">
+      <c r="E33" s="8" t="n">
         <v>-56448</v>
       </c>
-      <c r="F33" s="14" t="n">
+      <c r="F33" s="8" t="n">
         <v>-637915</v>
       </c>
-      <c r="G33" s="14" t="n">
-        <v>-600590.5449999999</v>
+      <c r="G33" s="8" t="n">
+        <v>1217667.982278481</v>
       </c>
     </row>
     <row r="34">
@@ -2401,7 +2401,7 @@
         <v>139640</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>143737</v>
+        <v>230321</v>
       </c>
     </row>
     <row r="37">
@@ -2426,32 +2426,32 @@
         <v>159640</v>
       </c>
       <c r="G37" s="8" t="n">
-        <v>163737</v>
+        <v>250321</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>✅ ЧИСТАЯ ПРИБЫЛЬ</t>
         </is>
       </c>
-      <c r="B38" s="14" t="n">
+      <c r="B38" s="8" t="n">
         <v>-513988</v>
       </c>
-      <c r="C38" s="14" t="n">
+      <c r="C38" s="8" t="n">
         <v>328010</v>
       </c>
-      <c r="D38" s="14" t="n">
+      <c r="D38" s="8" t="n">
         <v>-513988</v>
       </c>
-      <c r="E38" s="14" t="n">
+      <c r="E38" s="8" t="n">
         <v>-97589</v>
       </c>
-      <c r="F38" s="14" t="n">
+      <c r="F38" s="8" t="n">
         <v>-797555</v>
       </c>
-      <c r="G38" s="14" t="n">
-        <v>-764328</v>
+      <c r="G38" s="8" t="n">
+        <v>967347</v>
       </c>
     </row>
     <row r="39">
@@ -2467,7 +2467,7 @@
       <c r="F39" s="16" t="inlineStr"/>
       <c r="G39" s="16" t="inlineStr">
         <is>
-          <t>-25.3%</t>
+          <t>20.0%</t>
         </is>
       </c>
     </row>
@@ -2515,12 +2515,12 @@
     <row r="44">
       <c r="A44" s="17" t="inlineStr">
         <is>
-          <t>Требуемая выручка (новый контракт)</t>
+          <t>Цель: рент. чистой прибыли</t>
         </is>
       </c>
       <c r="B44" s="20" t="inlineStr">
         <is>
-          <t>3,018,478 ₽</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="C44" s="19" t="n"/>
@@ -2532,14 +2532,10 @@
     <row r="45">
       <c r="A45" s="17" t="inlineStr">
         <is>
-          <t>Прирост выручки</t>
-        </is>
-      </c>
-      <c r="B45" s="18" t="inlineStr">
-        <is>
-          <t>+783,814 ₽</t>
-        </is>
-      </c>
+          <t>──────────────────────────────</t>
+        </is>
+      </c>
+      <c r="B45" s="18" t="inlineStr"/>
       <c r="C45" s="19" t="n"/>
       <c r="D45" s="19" t="n"/>
       <c r="E45" s="19" t="n"/>
@@ -2549,12 +2545,12 @@
     <row r="46">
       <c r="A46" s="17" t="inlineStr">
         <is>
-          <t>Прирост контракта, %</t>
-        </is>
-      </c>
-      <c r="B46" s="18" t="inlineStr">
-        <is>
-          <t>+35.1%</t>
+          <t>Требуемая выручка (новый контракт)</t>
+        </is>
+      </c>
+      <c r="B46" s="20" t="inlineStr">
+        <is>
+          <t>4,836,736 ₽</t>
         </is>
       </c>
       <c r="C46" s="19" t="n"/>
@@ -2566,12 +2562,12 @@
     <row r="47">
       <c r="A47" s="17" t="inlineStr">
         <is>
-          <t>Требуемая МЕСЯЧНАЯ ставка</t>
-        </is>
-      </c>
-      <c r="B47" s="20" t="inlineStr">
-        <is>
-          <t>754,619 ₽/мес</t>
+          <t>Прирост выручки</t>
+        </is>
+      </c>
+      <c r="B47" s="18" t="inlineStr">
+        <is>
+          <t>+2,602,072 ₽</t>
         </is>
       </c>
       <c r="C47" s="19" t="n"/>
@@ -2583,12 +2579,12 @@
     <row r="48">
       <c r="A48" s="17" t="inlineStr">
         <is>
-          <t>Текущая МЕСЯЧНАЯ ставка</t>
+          <t>Прирост контракта, %</t>
         </is>
       </c>
       <c r="B48" s="18" t="inlineStr">
         <is>
-          <t>558,666 ₽/мес</t>
+          <t>+116.4%</t>
         </is>
       </c>
       <c r="C48" s="19" t="n"/>
@@ -2600,19 +2596,96 @@
     <row r="49">
       <c r="A49" s="17" t="inlineStr">
         <is>
-          <t>Рентабельность чистой прибыли</t>
-        </is>
-      </c>
-      <c r="B49" s="20" t="inlineStr">
-        <is>
-          <t>-25.3%</t>
-        </is>
-      </c>
+          <t>──────────────────────────────</t>
+        </is>
+      </c>
+      <c r="B49" s="18" t="inlineStr"/>
       <c r="C49" s="19" t="n"/>
       <c r="D49" s="19" t="n"/>
       <c r="E49" s="19" t="n"/>
       <c r="F49" s="19" t="n"/>
       <c r="G49" s="19" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>Требуемая МЕСЯЧНАЯ ставка</t>
+        </is>
+      </c>
+      <c r="B50" s="20" t="inlineStr">
+        <is>
+          <t>1,209,184 ₽/мес</t>
+        </is>
+      </c>
+      <c r="C50" s="19" t="n"/>
+      <c r="D50" s="19" t="n"/>
+      <c r="E50" s="19" t="n"/>
+      <c r="F50" s="19" t="n"/>
+      <c r="G50" s="19" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>Текущая МЕСЯЧНАЯ ставка</t>
+        </is>
+      </c>
+      <c r="B51" s="18" t="inlineStr">
+        <is>
+          <t>558,666 ₽/мес</t>
+        </is>
+      </c>
+      <c r="C51" s="19" t="n"/>
+      <c r="D51" s="19" t="n"/>
+      <c r="E51" s="19" t="n"/>
+      <c r="F51" s="19" t="n"/>
+      <c r="G51" s="19" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>Прирост мес. ставки</t>
+        </is>
+      </c>
+      <c r="B52" s="18" t="inlineStr">
+        <is>
+          <t>+650,518 ₽/мес</t>
+        </is>
+      </c>
+      <c r="C52" s="19" t="n"/>
+      <c r="D52" s="19" t="n"/>
+      <c r="E52" s="19" t="n"/>
+      <c r="F52" s="19" t="n"/>
+      <c r="G52" s="19" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t>──────────────────────────────</t>
+        </is>
+      </c>
+      <c r="B53" s="18" t="inlineStr"/>
+      <c r="C53" s="19" t="n"/>
+      <c r="D53" s="19" t="n"/>
+      <c r="E53" s="19" t="n"/>
+      <c r="F53" s="19" t="n"/>
+      <c r="G53" s="19" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>Рентабельность ЧП (сценарий)</t>
+        </is>
+      </c>
+      <c r="B54" s="20" t="inlineStr">
+        <is>
+          <t>20.0%</t>
+        </is>
+      </c>
+      <c r="C54" s="19" t="n"/>
+      <c r="D54" s="19" t="n"/>
+      <c r="E54" s="19" t="n"/>
+      <c r="F54" s="19" t="n"/>
+      <c r="G54" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2629,7 +2702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2644,7 +2717,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Финансовая модель — Астрид  |  Сценарий: ФОТ +40%</t>
+          <t>Финансовая модель — Астрид  |  ФОТ +40%  →  цель ЧП 20%</t>
         </is>
       </c>
     </row>
@@ -2766,7 +2839,7 @@
         <v>2234664</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>3279748.740000001</v>
+        <v>5167459.101265823</v>
       </c>
     </row>
     <row r="7">
@@ -3247,28 +3320,28 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>ВАЛОВАЯ ПРИБЫЛЬ</t>
         </is>
       </c>
-      <c r="B28" s="14" t="n">
+      <c r="B28" s="8" t="n">
         <v>-419488</v>
       </c>
-      <c r="C28" s="14" t="n">
+      <c r="C28" s="8" t="n">
         <v>454070</v>
       </c>
-      <c r="D28" s="14" t="n">
+      <c r="D28" s="8" t="n">
         <v>-419488</v>
       </c>
-      <c r="E28" s="14" t="n">
+      <c r="E28" s="8" t="n">
         <v>28471</v>
       </c>
-      <c r="F28" s="14" t="n">
+      <c r="F28" s="8" t="n">
         <v>-356435</v>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>-306669.0599999991</v>
+      <c r="G28" s="8" t="n">
+        <v>1581041.301265823</v>
       </c>
     </row>
     <row r="29">
@@ -3284,7 +3357,7 @@
       <c r="F29" s="16" t="inlineStr"/>
       <c r="G29" s="16" t="inlineStr">
         <is>
-          <t>-9.4%</t>
+          <t>30.6%</t>
         </is>
       </c>
     </row>
@@ -3352,28 +3425,28 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>ОПЕРАЦИОННАЯ ПРИБЫЛЬ</t>
         </is>
       </c>
-      <c r="B33" s="14" t="n">
+      <c r="B33" s="8" t="n">
         <v>-475309</v>
       </c>
-      <c r="C33" s="14" t="n">
+      <c r="C33" s="8" t="n">
         <v>369151</v>
       </c>
-      <c r="D33" s="14" t="n">
+      <c r="D33" s="8" t="n">
         <v>-475309</v>
       </c>
-      <c r="E33" s="14" t="n">
+      <c r="E33" s="8" t="n">
         <v>-56448</v>
       </c>
-      <c r="F33" s="14" t="n">
+      <c r="F33" s="8" t="n">
         <v>-637915</v>
       </c>
-      <c r="G33" s="14" t="n">
-        <v>-588149.0599999991</v>
+      <c r="G33" s="8" t="n">
+        <v>1299561.301265823</v>
       </c>
     </row>
     <row r="34">
@@ -3436,7 +3509,7 @@
         <v>139640</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>156179</v>
+        <v>246069</v>
       </c>
     </row>
     <row r="37">
@@ -3461,32 +3534,32 @@
         <v>159640</v>
       </c>
       <c r="G37" s="8" t="n">
-        <v>176179</v>
+        <v>266069</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>✅ ЧИСТАЯ ПРИБЫЛЬ</t>
         </is>
       </c>
-      <c r="B38" s="14" t="n">
+      <c r="B38" s="8" t="n">
         <v>-513988</v>
       </c>
-      <c r="C38" s="14" t="n">
+      <c r="C38" s="8" t="n">
         <v>328010</v>
       </c>
-      <c r="D38" s="14" t="n">
+      <c r="D38" s="8" t="n">
         <v>-513988</v>
       </c>
-      <c r="E38" s="14" t="n">
+      <c r="E38" s="8" t="n">
         <v>-97589</v>
       </c>
-      <c r="F38" s="14" t="n">
+      <c r="F38" s="8" t="n">
         <v>-797555</v>
       </c>
-      <c r="G38" s="14" t="n">
-        <v>-764328</v>
+      <c r="G38" s="8" t="n">
+        <v>1033492</v>
       </c>
     </row>
     <row r="39">
@@ -3502,7 +3575,7 @@
       <c r="F39" s="16" t="inlineStr"/>
       <c r="G39" s="16" t="inlineStr">
         <is>
-          <t>-23.3%</t>
+          <t>20.0%</t>
         </is>
       </c>
     </row>
@@ -3550,12 +3623,12 @@
     <row r="44">
       <c r="A44" s="17" t="inlineStr">
         <is>
-          <t>Требуемая выручка (новый контракт)</t>
+          <t>Цель: рент. чистой прибыли</t>
         </is>
       </c>
       <c r="B44" s="20" t="inlineStr">
         <is>
-          <t>3,279,749 ₽</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="C44" s="19" t="n"/>
@@ -3567,14 +3640,10 @@
     <row r="45">
       <c r="A45" s="17" t="inlineStr">
         <is>
-          <t>Прирост выручки</t>
-        </is>
-      </c>
-      <c r="B45" s="18" t="inlineStr">
-        <is>
-          <t>+1,045,085 ₽</t>
-        </is>
-      </c>
+          <t>──────────────────────────────</t>
+        </is>
+      </c>
+      <c r="B45" s="18" t="inlineStr"/>
       <c r="C45" s="19" t="n"/>
       <c r="D45" s="19" t="n"/>
       <c r="E45" s="19" t="n"/>
@@ -3584,12 +3653,12 @@
     <row r="46">
       <c r="A46" s="17" t="inlineStr">
         <is>
-          <t>Прирост контракта, %</t>
-        </is>
-      </c>
-      <c r="B46" s="18" t="inlineStr">
-        <is>
-          <t>+46.8%</t>
+          <t>Требуемая выручка (новый контракт)</t>
+        </is>
+      </c>
+      <c r="B46" s="20" t="inlineStr">
+        <is>
+          <t>5,167,459 ₽</t>
         </is>
       </c>
       <c r="C46" s="19" t="n"/>
@@ -3601,12 +3670,12 @@
     <row r="47">
       <c r="A47" s="17" t="inlineStr">
         <is>
-          <t>Требуемая МЕСЯЧНАЯ ставка</t>
-        </is>
-      </c>
-      <c r="B47" s="20" t="inlineStr">
-        <is>
-          <t>819,937 ₽/мес</t>
+          <t>Прирост выручки</t>
+        </is>
+      </c>
+      <c r="B47" s="18" t="inlineStr">
+        <is>
+          <t>+2,932,795 ₽</t>
         </is>
       </c>
       <c r="C47" s="19" t="n"/>
@@ -3618,12 +3687,12 @@
     <row r="48">
       <c r="A48" s="17" t="inlineStr">
         <is>
-          <t>Текущая МЕСЯЧНАЯ ставка</t>
+          <t>Прирост контракта, %</t>
         </is>
       </c>
       <c r="B48" s="18" t="inlineStr">
         <is>
-          <t>558,666 ₽/мес</t>
+          <t>+131.2%</t>
         </is>
       </c>
       <c r="C48" s="19" t="n"/>
@@ -3635,19 +3704,96 @@
     <row r="49">
       <c r="A49" s="17" t="inlineStr">
         <is>
-          <t>Рентабельность чистой прибыли</t>
-        </is>
-      </c>
-      <c r="B49" s="20" t="inlineStr">
-        <is>
-          <t>-23.3%</t>
-        </is>
-      </c>
+          <t>──────────────────────────────</t>
+        </is>
+      </c>
+      <c r="B49" s="18" t="inlineStr"/>
       <c r="C49" s="19" t="n"/>
       <c r="D49" s="19" t="n"/>
       <c r="E49" s="19" t="n"/>
       <c r="F49" s="19" t="n"/>
       <c r="G49" s="19" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>Требуемая МЕСЯЧНАЯ ставка</t>
+        </is>
+      </c>
+      <c r="B50" s="20" t="inlineStr">
+        <is>
+          <t>1,291,865 ₽/мес</t>
+        </is>
+      </c>
+      <c r="C50" s="19" t="n"/>
+      <c r="D50" s="19" t="n"/>
+      <c r="E50" s="19" t="n"/>
+      <c r="F50" s="19" t="n"/>
+      <c r="G50" s="19" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>Текущая МЕСЯЧНАЯ ставка</t>
+        </is>
+      </c>
+      <c r="B51" s="18" t="inlineStr">
+        <is>
+          <t>558,666 ₽/мес</t>
+        </is>
+      </c>
+      <c r="C51" s="19" t="n"/>
+      <c r="D51" s="19" t="n"/>
+      <c r="E51" s="19" t="n"/>
+      <c r="F51" s="19" t="n"/>
+      <c r="G51" s="19" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>Прирост мес. ставки</t>
+        </is>
+      </c>
+      <c r="B52" s="18" t="inlineStr">
+        <is>
+          <t>+733,199 ₽/мес</t>
+        </is>
+      </c>
+      <c r="C52" s="19" t="n"/>
+      <c r="D52" s="19" t="n"/>
+      <c r="E52" s="19" t="n"/>
+      <c r="F52" s="19" t="n"/>
+      <c r="G52" s="19" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t>──────────────────────────────</t>
+        </is>
+      </c>
+      <c r="B53" s="18" t="inlineStr"/>
+      <c r="C53" s="19" t="n"/>
+      <c r="D53" s="19" t="n"/>
+      <c r="E53" s="19" t="n"/>
+      <c r="F53" s="19" t="n"/>
+      <c r="G53" s="19" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>Рентабельность ЧП (сценарий)</t>
+        </is>
+      </c>
+      <c r="B54" s="20" t="inlineStr">
+        <is>
+          <t>20.0%</t>
+        </is>
+      </c>
+      <c r="C54" s="19" t="n"/>
+      <c r="D54" s="19" t="n"/>
+      <c r="E54" s="19" t="n"/>
+      <c r="F54" s="19" t="n"/>
+      <c r="G54" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>